<commit_message>
feat: Add financial routing and scheme-based facility suggestions - Implement new routing module (src/resilicare/routing.py) with simulated facility data. - Update demo server to expose a route preview endpoint and include routing assessments. - Enhance demo UI to display patient schemes and provide a route preview button. - Append 'scheme' attribute to the simulated patient datasets. - Add tests for the routing module and extend existing audit server tests. - Update README.md and module exports to include the new routing capabilities.
</commit_message>
<xml_diff>
--- a/data/PatientTriage_Simulated_Dataset.xlsx
+++ b/data/PatientTriage_Simulated_Dataset.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Patients" sheetId="1" r:id="R2efa584f21934cf7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="2" r:id="Rc021ad1a724c4f88"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codebook" sheetId="3" r:id="R73123fdab1b34a26"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Label Guidance" sheetId="4" r:id="R0420360b433d4b4b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Patients" sheetId="1" r:id="R7880bbea949c4bc1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="2" r:id="R0b316b23f2e14b68"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codebook" sheetId="3" r:id="R96f9a3190009440b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Label Guidance" sheetId="4" r:id="R33e3abfac31a4436"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -21,7 +21,7 @@
     <x:numFmt numFmtId="201" formatCode="0.0"/>
     <x:numFmt numFmtId="202" formatCode="0"/>
   </x:numFmts>
-  <x:fonts count="7">
+  <x:fonts count="8">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -62,8 +62,13 @@
       <x:color rgb="FF991B1B"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF172B3A"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="7">
+  <x:fills count="11">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -93,6 +98,26 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFEE2E2"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEDE9FE"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEDE9FE"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -192,7 +217,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="69">
+  <x:cellXfs count="77">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -419,6 +444,22 @@
     <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -432,7 +473,7 @@
         <x:color rgb="FFFFFFFF"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFB91C1C"/>
         </x:patternFill>
       </x:fill>
@@ -443,7 +484,7 @@
         <x:color rgb="FFFFFFFF"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEA580C"/>
         </x:patternFill>
       </x:fill>
@@ -454,7 +495,7 @@
         <x:color rgb="FF111827"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFACC15"/>
         </x:patternFill>
       </x:fill>
@@ -465,7 +506,7 @@
         <x:color rgb="FFFFFFFF"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FF22C55E"/>
         </x:patternFill>
       </x:fill>
@@ -476,7 +517,7 @@
         <x:color rgb="FFFFFFFF"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FF2563EB"/>
         </x:patternFill>
       </x:fill>
@@ -487,7 +528,7 @@
         <x:color rgb="FF166534"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDCFCE7"/>
         </x:patternFill>
       </x:fill>
@@ -498,7 +539,7 @@
         <x:color rgb="FF991B1B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -794,11 +835,12 @@
     <x:col min="31" max="31" width="36" hidden="0" customWidth="1"/>
     <x:col min="32" max="32" width="22" hidden="0" customWidth="1"/>
     <x:col min="33" max="33" width="18" hidden="0" customWidth="1"/>
+    <x:col min="34" max="34" width="16.8799991607666" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
       <x:c r="A1" s="4" t="str">
-        <x:v>ResiliCare - Synthetic Patient Triage Dataset v1.0</x:v>
+        <x:v>ResiliCare Synthetic Patient Triage Dataset · v1.1</x:v>
       </x:c>
       <x:c r="B1" s="4"/>
       <x:c r="C1" s="4"/>
@@ -970,6 +1012,9 @@
       <x:c r="AG4" s="20" t="str">
         <x:v>reassessment_scenario</x:v>
       </x:c>
+      <x:c r="AH4" t="str">
+        <x:v>scheme</x:v>
+      </x:c>
     </x:row>
     <x:row r="5" ht="72" customHeight="1">
       <x:c r="A5" s="35" t="str">
@@ -1057,6 +1102,9 @@
       <x:c r="AG5" s="41" t="b">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="AH5" t="str">
+        <x:v>PM-JAY</x:v>
+      </x:c>
     </x:row>
     <x:row r="6" ht="72" customHeight="1">
       <x:c r="A6" s="35" t="str">
@@ -1156,6 +1204,9 @@
       <x:c r="AG6" s="41" t="b">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="AH6" t="str">
+        <x:v>ESIC</x:v>
+      </x:c>
     </x:row>
     <x:row r="7" ht="72" customHeight="1">
       <x:c r="A7" s="35" t="str">
@@ -1255,6 +1306,9 @@
       <x:c r="AG7" s="41" t="b">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="AH7" t="str">
+        <x:v>Private Insurer X</x:v>
+      </x:c>
     </x:row>
     <x:row r="8" ht="72" customHeight="1">
       <x:c r="A8" s="35" t="str">
@@ -1354,6 +1408,9 @@
       <x:c r="AG8" s="41" t="b">
         <x:v>1</x:v>
       </x:c>
+      <x:c r="AH8" t="str">
+        <x:v>Self-pay</x:v>
+      </x:c>
     </x:row>
     <x:row r="9" ht="72" customHeight="1">
       <x:c r="A9" s="35" t="str">
@@ -1453,6 +1510,9 @@
       <x:c r="AG9" s="41" t="b">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="AH9" t="str">
+        <x:v>PM-JAY</x:v>
+      </x:c>
     </x:row>
     <x:row r="10" ht="72" customHeight="1">
       <x:c r="A10" s="35" t="str">
@@ -1550,6 +1610,9 @@
       <x:c r="AG10" s="41" t="b">
         <x:v>1</x:v>
       </x:c>
+      <x:c r="AH10" t="str">
+        <x:v>ESIC</x:v>
+      </x:c>
     </x:row>
     <x:row r="11" ht="72" customHeight="1">
       <x:c r="A11" s="35" t="str">
@@ -1649,6 +1712,9 @@
       <x:c r="AG11" s="41" t="b">
         <x:v>1</x:v>
       </x:c>
+      <x:c r="AH11" t="str">
+        <x:v>Private Insurer X</x:v>
+      </x:c>
     </x:row>
     <x:row r="12" ht="72" customHeight="1">
       <x:c r="A12" s="35" t="str">
@@ -1748,6 +1814,9 @@
       <x:c r="AG12" s="41" t="b">
         <x:v>1</x:v>
       </x:c>
+      <x:c r="AH12" t="str">
+        <x:v>Self-pay</x:v>
+      </x:c>
     </x:row>
     <x:row r="13" ht="72" customHeight="1">
       <x:c r="A13" s="35" t="str">
@@ -1849,6 +1918,9 @@
       <x:c r="AG13" s="41" t="b">
         <x:v>1</x:v>
       </x:c>
+      <x:c r="AH13" t="str">
+        <x:v>PM-JAY</x:v>
+      </x:c>
     </x:row>
     <x:row r="14" ht="72" customHeight="1">
       <x:c r="A14" s="35" t="str">
@@ -1950,6 +2022,9 @@
       <x:c r="AG14" s="41" t="b">
         <x:v>1</x:v>
       </x:c>
+      <x:c r="AH14" t="str">
+        <x:v>ESIC</x:v>
+      </x:c>
     </x:row>
     <x:row r="15" ht="72" customHeight="1">
       <x:c r="A15" s="35" t="str">
@@ -2051,6 +2126,9 @@
       <x:c r="AG15" s="41" t="b">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="AH15" t="str">
+        <x:v>Private Insurer X</x:v>
+      </x:c>
     </x:row>
     <x:row r="16" ht="72" customHeight="1">
       <x:c r="A16" s="35" t="str">
@@ -2152,6 +2230,9 @@
       <x:c r="AG16" s="41" t="b">
         <x:v>1</x:v>
       </x:c>
+      <x:c r="AH16" t="str">
+        <x:v>Self-pay</x:v>
+      </x:c>
     </x:row>
     <x:row r="17" ht="72" customHeight="1">
       <x:c r="A17" s="35" t="str">
@@ -2253,6 +2334,9 @@
       <x:c r="AG17" s="41" t="b">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="AH17" t="str">
+        <x:v>PM-JAY</x:v>
+      </x:c>
     </x:row>
     <x:row r="18" ht="72" customHeight="1">
       <x:c r="A18" s="35" t="str">
@@ -2354,6 +2438,9 @@
       <x:c r="AG18" s="41" t="b">
         <x:v>1</x:v>
       </x:c>
+      <x:c r="AH18" t="str">
+        <x:v>ESIC</x:v>
+      </x:c>
     </x:row>
     <x:row r="19" ht="72" customHeight="1">
       <x:c r="A19" s="35" t="str">
@@ -2455,6 +2542,9 @@
       <x:c r="AG19" s="41" t="b">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="AH19" t="str">
+        <x:v>PM-JAY</x:v>
+      </x:c>
     </x:row>
     <x:row r="20" ht="72" customHeight="1">
       <x:c r="A20" s="35" t="str">
@@ -2556,6 +2646,9 @@
       <x:c r="AG20" s="41" t="b">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="AH20" t="str">
+        <x:v>ESIC</x:v>
+      </x:c>
     </x:row>
     <x:row r="21" ht="72" customHeight="1">
       <x:c r="A21" s="35" t="str">
@@ -2657,6 +2750,9 @@
       <x:c r="AG21" s="41" t="b">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="AH21" t="str">
+        <x:v>Private Insurer X</x:v>
+      </x:c>
     </x:row>
     <x:row r="22" ht="72" customHeight="1">
       <x:c r="A22" s="35" t="str">
@@ -2758,6 +2854,9 @@
       <x:c r="AG22" s="41" t="b">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="AH22" t="str">
+        <x:v>Self-pay</x:v>
+      </x:c>
     </x:row>
     <x:row r="23" ht="72" customHeight="1">
       <x:c r="A23" s="35" t="str">
@@ -2859,6 +2958,9 @@
       <x:c r="AG23" s="41" t="b">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="AH23" t="str">
+        <x:v>PM-JAY</x:v>
+      </x:c>
     </x:row>
     <x:row r="24" ht="72" customHeight="1">
       <x:c r="A24" s="42" t="str">
@@ -2959,6 +3061,9 @@
       </x:c>
       <x:c r="AG24" s="48" t="b">
         <x:v>1</x:v>
+      </x:c>
+      <x:c r="AH24" t="str">
+        <x:v>Private Insurer X</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2983,9 +3088,14 @@
       <x:formula>5</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
+  <x:dataValidations count="1">
+    <x:dataValidation type="list" sqref="AH5:AH24">
+      <x:formula1>"PM-JAY,ESIC,Private Insurer X,Self-pay"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R89f2d5f355594750"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0850e9b367a54681"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3271,7 +3381,7 @@
   <x:cols>
     <x:col min="1" max="1" width="34" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="20" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="24" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="32.5" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="66" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
@@ -3715,6 +3825,20 @@
       <x:c r="C36" s="44" t="str"/>
       <x:c r="D36" s="60" t="str">
         <x:v>Candidate for later waiting-room/reassessment simulation</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="31.5" customHeight="1">
+      <x:c r="A37" t="str">
+        <x:v>scheme</x:v>
+      </x:c>
+      <x:c r="B37" t="str">
+        <x:v>enum</x:v>
+      </x:c>
+      <x:c r="C37" s="53" t="str">
+        <x:v>PM-JAY | ESIC | Private Insurer X | Self-pay</x:v>
+      </x:c>
+      <x:c r="D37" t="str">
+        <x:v>Synthetic coverage category for Task 13; not verified eligibility</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3791,6 +3915,14 @@
         <x:v>https://www.ena.org/education/emergency-nursing-triage-education-program/triage-portfolio</x:v>
       </x:c>
     </x:row>
+    <x:row r="9" ht="36" customHeight="1">
+      <x:c r="A9" s="75" t="str">
+        <x:v>Task 13 data</x:v>
+      </x:c>
+      <x:c r="B9" s="76" t="str">
+        <x:v>All scheme, eligibility, facility, distance, cashless, and room-rent values are simulated. No live NHCX or insurer lookup is performed.</x:v>
+      </x:c>
+    </x:row>
     <x:row r="10">
       <x:c r="A10" s="68" t="str">
         <x:v>Before using these labels in judging materials, obtain documented review and record reviewer role, date, accepted level, and any change rationale in a separate versioned review file.</x:v>

</xml_diff>